<commit_message>
test(oracle): recalcular escenarios con mercado y consecuencias auditados
</commit_message>
<xml_diff>
--- a/tests/oracle/ORACULO_SIDE.xlsx
+++ b/tests/oracle/ORACULO_SIDE.xlsx
@@ -3720,11 +3720,11 @@
         </is>
       </c>
       <c r="D7" s="186">
-        <f>B9&gt;B10</f>
+        <f>B11&gt;B10</f>
         <v/>
       </c>
       <c r="E7" s="186">
-        <f>IF(D7,0.25*B13*MIN(1,IFERROR((B9-B10)/B10,0)),0)</f>
+        <f>IF(D7,0.25*B13*MIN(1,IFERROR((B11-B10)/B10,0)),0)</f>
         <v/>
       </c>
       <c r="F7" s="186">

</xml_diff>